<commit_message>
phase-5.8: incorporate expert follow-up workbook
</commit_message>
<xml_diff>
--- a/data/human_judgment/evaluators/expert_01/source/expert_01_blind_raw.xlsx
+++ b/data/human_judgment/evaluators/expert_01/source/expert_01_blind_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/furnari/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24B24442-A9BD-5045-A30A-2A005DE62C77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B59FDBEB-C432-D34D-977C-646B27473E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="27140" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="103">
   <si>
     <t>Validazione esperta dei syllabus — istruzioni (protocollo blind)</t>
   </si>
@@ -279,9 +279,6 @@
     <t>i prerequisiti sono stringati e fanno riferimento a specifici corsi</t>
   </si>
   <si>
-    <t>il mapping c'è, ma forse potrebbe essere un po' più dettagliato (es. sulle parti pratiche)</t>
-  </si>
-  <si>
     <t>Non c'è una struttura a blocchi, ma c'è da dire che le nostre istruzioni date ai docenti chiedevano di fare un ragionamento discorsivo, più che di suddividere a blocchi</t>
   </si>
   <si>
@@ -306,9 +303,6 @@
     <t>I contenuti del corso sono una lista di argomenti e manca una narrazione discorsiva dei contenuti e come questi contribuiscono ai risultati di apprendimento</t>
   </si>
   <si>
-    <t>Non si evince un mapping</t>
-  </si>
-  <si>
     <t>Modalità di verifica presenti e articolate in prove criteri.</t>
   </si>
   <si>
@@ -321,9 +315,6 @@
     <t>I prerequisiti sono sintetici ma adeguati</t>
   </si>
   <si>
-    <t>Il collegamento con i RA c'è ma potrebbe essere più esplicito.</t>
-  </si>
-  <si>
     <t>I contenuti sono un misto tra discorsivo ed elenco. Potrebbe essere organizzato meglio.</t>
   </si>
   <si>
@@ -333,9 +324,6 @@
     <t>Potrebbe essere più estesa, ma può anche andare bene così.</t>
   </si>
   <si>
-    <t>Il collegamento è solo implicito</t>
-  </si>
-  <si>
     <t>Potrebbero essere indicati in maniera più discorsiva</t>
   </si>
   <si>
@@ -360,13 +348,13 @@
     <t>I contenuti del corso potrebbero essere maggiormente articolati</t>
   </si>
   <si>
-    <t>Link implicito</t>
-  </si>
-  <si>
     <t>Si potrebbero inserire anche prerequisiti più generici (es. basi della programmazione)</t>
   </si>
   <si>
     <t>Ci sono dei simboli refusi ("--&gt;") [che so essere dovuti al portale e non sono riuscito a rimuovere]</t>
+  </si>
+  <si>
+    <t>Non è specificato come le due prove contribuiscono al voto finale. Non c'è la griglia di valutazione.</t>
   </si>
 </sst>
 </file>
@@ -1153,12 +1141,10 @@
         <v>55</v>
       </c>
       <c r="E10" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="8"/>
-      <c r="G10" s="8" t="s">
-        <v>77</v>
-      </c>
+      <c r="G10" s="8"/>
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" ht="108" customHeight="1" x14ac:dyDescent="0.2">
@@ -1179,7 +1165,7 @@
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H11" s="8"/>
     </row>
@@ -1221,7 +1207,7 @@
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H13" s="8"/>
     </row>
@@ -1342,7 +1328,7 @@
       </c>
       <c r="F5" s="8"/>
       <c r="G5" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H5" s="8"/>
     </row>
@@ -1364,7 +1350,7 @@
       </c>
       <c r="F6" s="8"/>
       <c r="G6" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H6" s="8"/>
     </row>
@@ -1386,7 +1372,7 @@
       </c>
       <c r="F7" s="8"/>
       <c r="G7" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H7" s="8"/>
     </row>
@@ -1428,7 +1414,7 @@
       </c>
       <c r="F9" s="8"/>
       <c r="G9" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H9" s="8"/>
     </row>
@@ -1446,12 +1432,10 @@
         <v>55</v>
       </c>
       <c r="E10" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="8"/>
-      <c r="G10" s="8" t="s">
-        <v>86</v>
-      </c>
+      <c r="G10" s="8"/>
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" ht="108" customHeight="1" x14ac:dyDescent="0.2">
@@ -1472,7 +1456,7 @@
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H11" s="8"/>
     </row>
@@ -1494,7 +1478,7 @@
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H12" s="8"/>
     </row>
@@ -1516,10 +1500,10 @@
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1659,7 +1643,7 @@
       </c>
       <c r="F6" s="8"/>
       <c r="G6" s="8" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H6" s="8"/>
     </row>
@@ -1721,7 +1705,7 @@
       </c>
       <c r="F9" s="8"/>
       <c r="G9" s="8" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="H9" s="8"/>
     </row>
@@ -1739,12 +1723,10 @@
         <v>55</v>
       </c>
       <c r="E10" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="8"/>
-      <c r="G10" s="8" t="s">
-        <v>91</v>
-      </c>
+      <c r="G10" s="8"/>
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" ht="108" customHeight="1" x14ac:dyDescent="0.2">
@@ -1765,7 +1747,7 @@
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="8" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="H11" s="8"/>
     </row>
@@ -1807,7 +1789,7 @@
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H13" s="8"/>
     </row>
@@ -2008,7 +1990,7 @@
       </c>
       <c r="F9" s="8"/>
       <c r="G9" s="8" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H9" s="8"/>
     </row>
@@ -2026,12 +2008,10 @@
         <v>55</v>
       </c>
       <c r="E10" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="8"/>
-      <c r="G10" s="8" t="s">
-        <v>95</v>
-      </c>
+      <c r="G10" s="8"/>
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" ht="108" customHeight="1" x14ac:dyDescent="0.2">
@@ -2052,7 +2032,7 @@
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="8" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="H11" s="8"/>
     </row>
@@ -2233,7 +2213,7 @@
       </c>
       <c r="F6" s="8"/>
       <c r="G6" s="8" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H6" s="8"/>
     </row>
@@ -2295,7 +2275,7 @@
       </c>
       <c r="F9" s="8"/>
       <c r="G9" s="8" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="H9" s="8"/>
     </row>
@@ -2313,10 +2293,12 @@
         <v>55</v>
       </c>
       <c r="E10" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
+      <c r="G10" s="8" t="s">
+        <v>102</v>
+      </c>
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" ht="108" customHeight="1" x14ac:dyDescent="0.2">
@@ -2337,7 +2319,7 @@
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="8" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="H11" s="8"/>
     </row>
@@ -2359,7 +2341,7 @@
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="8" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="H12" s="8"/>
     </row>
@@ -2381,10 +2363,10 @@
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -2600,12 +2582,10 @@
         <v>55</v>
       </c>
       <c r="E10" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="8"/>
-      <c r="G10" s="8" t="s">
-        <v>104</v>
-      </c>
+      <c r="G10" s="8"/>
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" ht="108" customHeight="1" x14ac:dyDescent="0.2">
@@ -2626,7 +2606,7 @@
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="8" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="H11" s="8"/>
     </row>
@@ -2867,7 +2847,7 @@
       </c>
       <c r="F9" s="8"/>
       <c r="G9" s="8" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H9" s="8"/>
     </row>
@@ -2949,7 +2929,7 @@
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="H13" s="8"/>
     </row>
@@ -3065,7 +3045,9 @@
       <c r="D5" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="7"/>
+      <c r="E5" s="7">
+        <v>2</v>
+      </c>
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
       <c r="H5" s="8"/>
@@ -3083,7 +3065,9 @@
       <c r="D6" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="7"/>
+      <c r="E6" s="7">
+        <v>2</v>
+      </c>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
@@ -3101,7 +3085,9 @@
       <c r="D7" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="7"/>
+      <c r="E7" s="7">
+        <v>2</v>
+      </c>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
@@ -3119,7 +3105,9 @@
       <c r="D8" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="E8" s="7"/>
+      <c r="E8" s="7">
+        <v>2</v>
+      </c>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
@@ -3137,7 +3125,9 @@
       <c r="D9" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="7"/>
+      <c r="E9" s="7">
+        <v>2</v>
+      </c>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
@@ -3155,7 +3145,9 @@
       <c r="D10" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E10" s="7"/>
+      <c r="E10" s="7">
+        <v>2</v>
+      </c>
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
@@ -3173,7 +3165,9 @@
       <c r="D11" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="E11" s="7"/>
+      <c r="E11" s="7">
+        <v>2</v>
+      </c>
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
@@ -3191,7 +3185,9 @@
       <c r="D12" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E12" s="7"/>
+      <c r="E12" s="7">
+        <v>2</v>
+      </c>
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
@@ -3209,7 +3205,9 @@
       <c r="D13" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="E13" s="7"/>
+      <c r="E13" s="7">
+        <v>2</v>
+      </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>

</xml_diff>